<commit_message>
Add quartz angle frequency scatter and trend analysis
</commit_message>
<xml_diff>
--- a/He-Ne 激光的纵横模分析和模分裂/lab_report/实验数据第二次.xlsx
+++ b/He-Ne 激光的纵横模分析和模分裂/lab_report/实验数据第二次.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HONOR\Documents\Codex\lab_report\He-Ne 激光的纵横模分析和模分裂\lab_report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A227A97-A22E-4434-A577-D61DBC227DD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA16045D-3AE4-45AC-82DA-7E5C7508C322}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="23236" windowHeight="13875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4330" yWindow="2010" windowWidth="19200" windowHeight="9970" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>出光带宽</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -53,6 +53,34 @@
   </si>
   <si>
     <t>νFSR</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>偏振片转过的角度</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>一峰相对电位</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>二峰相对点位</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>晶片转角（2.2为垂直时示数）</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>左峰</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>右峰</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>差值</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -758,42 +786,42 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet1!$F$24:$F$34</c:f>
+              <c:f>Sheet1!$D$24:$D$34</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="11"/>
                 <c:pt idx="0">
-                  <c:v>1.2250000000000001</c:v>
+                  <c:v>1.25</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.4499999999999997</c:v>
+                  <c:v>1.4999999999999996</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.3250000000000002</c:v>
+                  <c:v>1.4000000000000001</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1.4000000000000004</c:v>
+                  <c:v>1.4500000000000002</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1.1749999999999998</c:v>
+                  <c:v>1.2499999999999996</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1.35</c:v>
+                  <c:v>1.4500000000000002</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1.3750000000000002</c:v>
+                  <c:v>1.5000000000000004</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1.4</c:v>
+                  <c:v>1.5</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.72499999999999987</c:v>
+                  <c:v>0.75</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.57500000000000018</c:v>
+                  <c:v>0.65000000000000036</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.75000000000000022</c:v>
+                  <c:v>0.75</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2445,14 +2473,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F43"/>
-  <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="23.58203125" customWidth="1"/>
+    <col min="2" max="2" width="12.33203125" customWidth="1"/>
+    <col min="3" max="3" width="11.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
         <v>1</v>
       </c>
@@ -2466,7 +2499,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>1</v>
       </c>
@@ -2488,7 +2521,7 @@
         <v>1138.4822134387352</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2</v>
       </c>
@@ -2510,7 +2543,7 @@
         <v>1054.1501976284585</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>3</v>
       </c>
@@ -2528,17 +2561,28 @@
         <v>2667</v>
       </c>
       <c r="F5">
-        <f t="shared" ref="F4:F5" si="1">E5*(B5-C5)/D5</f>
+        <f t="shared" ref="F5" si="1">E5*(B5-C5)/D5</f>
         <v>1117.3992094861653</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="F6">
         <f>AVERAGE(F3:F5)</f>
         <v>1103.3438735177863</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>0</v>
       </c>
@@ -2549,7 +2593,7 @@
         <v>-2.4329999999999998</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>15</v>
       </c>
@@ -2560,7 +2604,7 @@
         <v>-2.766</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>30</v>
       </c>
@@ -2571,7 +2615,7 @@
         <v>-3.0830000000000002</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>45</v>
       </c>
@@ -2582,7 +2626,7 @@
         <v>-3.1</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>60</v>
       </c>
@@ -2593,7 +2637,7 @@
         <v>-3.3660000000000001</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>75</v>
       </c>
@@ -2604,7 +2648,7 @@
         <v>-3.6659999999999999</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>90</v>
       </c>
@@ -2615,7 +2659,7 @@
         <v>-3.65</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>105</v>
       </c>
@@ -2626,7 +2670,7 @@
         <v>-3.4159999999999999</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>120</v>
       </c>
@@ -2637,7 +2681,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>135</v>
       </c>
@@ -2648,7 +2692,7 @@
         <v>-2.6</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>150</v>
       </c>
@@ -2659,7 +2703,7 @@
         <v>-2.383</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>165</v>
       </c>
@@ -2670,7 +2714,7 @@
         <v>-2.35</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>180</v>
       </c>
@@ -2681,7 +2725,21 @@
         <v>-2.4</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>8</v>
+      </c>
+      <c r="B23" t="s">
+        <v>9</v>
+      </c>
+      <c r="C23" t="s">
+        <v>10</v>
+      </c>
+      <c r="D23" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>2.2000000000000002</v>
       </c>
@@ -2692,17 +2750,11 @@
         <v>-3.8</v>
       </c>
       <c r="D24">
-        <v>1.9</v>
-      </c>
-      <c r="E24">
-        <v>3.1</v>
-      </c>
-      <c r="F24">
-        <f>(E24+C24-D24-B24)/2</f>
-        <v>1.2250000000000001</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.4">
+        <f t="shared" ref="D24:D43" si="2">(+C24-B24)</f>
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>3.2</v>
       </c>
@@ -2713,17 +2765,11 @@
         <v>-3.35</v>
       </c>
       <c r="D25">
-        <v>2.1</v>
-      </c>
-      <c r="E25">
-        <v>3.5</v>
-      </c>
-      <c r="F25">
-        <f t="shared" ref="F25:F34" si="2">(E25+C25-D25-B25)/2</f>
-        <v>1.4499999999999997</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.4">
+        <f t="shared" si="2"/>
+        <v>1.4999999999999996</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>4.2</v>
       </c>
@@ -2734,17 +2780,11 @@
         <v>-1.8</v>
       </c>
       <c r="D26">
-        <v>3.55</v>
-      </c>
-      <c r="E26">
-        <v>4.8</v>
-      </c>
-      <c r="F26">
         <f t="shared" si="2"/>
-        <v>1.3250000000000002</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.4">
+        <v>1.4000000000000001</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>5.2</v>
       </c>
@@ -2755,17 +2795,11 @@
         <v>-2.0499999999999998</v>
       </c>
       <c r="D27">
-        <v>3.3</v>
-      </c>
-      <c r="E27">
-        <v>4.6500000000000004</v>
-      </c>
-      <c r="F27">
         <f t="shared" si="2"/>
-        <v>1.4000000000000004</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.4">
+        <v>1.4500000000000002</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>6.2</v>
       </c>
@@ -2776,17 +2810,11 @@
         <v>-3.1</v>
       </c>
       <c r="D28">
-        <v>2.5499999999999998</v>
-      </c>
-      <c r="E28">
-        <v>3.65</v>
-      </c>
-      <c r="F28">
         <f t="shared" si="2"/>
-        <v>1.1749999999999998</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.4">
+        <v>1.2499999999999996</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>7.2</v>
       </c>
@@ -2797,17 +2825,11 @@
         <v>-3</v>
       </c>
       <c r="D29">
-        <v>2.5</v>
-      </c>
-      <c r="E29">
-        <v>3.75</v>
-      </c>
-      <c r="F29">
         <f t="shared" si="2"/>
-        <v>1.35</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.4">
+        <v>1.4500000000000002</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>8.1999999999999993</v>
       </c>
@@ -2818,17 +2840,11 @@
         <v>-3.4</v>
       </c>
       <c r="D30">
-        <v>2.15</v>
-      </c>
-      <c r="E30">
-        <v>3.4</v>
-      </c>
-      <c r="F30">
         <f t="shared" si="2"/>
-        <v>1.3750000000000002</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.4">
+        <v>1.5000000000000004</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>9.1999999999999993</v>
       </c>
@@ -2839,134 +2855,188 @@
         <v>-4.75</v>
       </c>
       <c r="D31">
-        <v>0.95</v>
-      </c>
-      <c r="E31">
-        <v>2.25</v>
-      </c>
-      <c r="F31">
+        <f t="shared" si="2"/>
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A32">
+        <v>10.199999999999999</v>
+      </c>
+      <c r="B32">
+        <v>-4.9000000000000004</v>
+      </c>
+      <c r="C32">
+        <v>-4.1500000000000004</v>
+      </c>
+      <c r="D32">
+        <f t="shared" si="2"/>
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A33">
+        <v>11.2</v>
+      </c>
+      <c r="B33">
+        <v>8.25</v>
+      </c>
+      <c r="C33">
+        <v>8.9</v>
+      </c>
+      <c r="D33">
+        <f t="shared" si="2"/>
+        <v>0.65000000000000036</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A34">
+        <v>12.2</v>
+      </c>
+      <c r="B34">
+        <v>1.9</v>
+      </c>
+      <c r="C34">
+        <v>2.65</v>
+      </c>
+      <c r="D34">
+        <f t="shared" si="2"/>
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A35">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="B35">
+        <v>-4.5999999999999996</v>
+      </c>
+      <c r="C35">
+        <v>-4.4000000000000004</v>
+      </c>
+      <c r="D35">
+        <f>(+C35-B35)</f>
+        <v>0.19999999999999929</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A36">
+        <v>2.4</v>
+      </c>
+      <c r="B36">
+        <v>1.75</v>
+      </c>
+      <c r="C36">
+        <v>2.85</v>
+      </c>
+      <c r="D36">
+        <f t="shared" si="2"/>
+        <v>1.1000000000000001</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A37">
+        <v>2.6</v>
+      </c>
+      <c r="B37">
+        <v>2.1</v>
+      </c>
+      <c r="C37">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="D37">
+        <f t="shared" si="2"/>
+        <v>0.19999999999999973</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A38">
+        <v>2.8</v>
+      </c>
+      <c r="B38">
+        <v>-5.4</v>
+      </c>
+      <c r="C38">
+        <v>-4.2</v>
+      </c>
+      <c r="D38">
+        <f t="shared" si="2"/>
+        <v>1.2000000000000002</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A39">
+        <v>2.9</v>
+      </c>
+      <c r="B39">
+        <v>-4.9000000000000004</v>
+      </c>
+      <c r="C39">
+        <v>-3.45</v>
+      </c>
+      <c r="D39">
+        <f t="shared" si="2"/>
+        <v>1.4500000000000002</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A40">
+        <v>3</v>
+      </c>
+      <c r="B40">
+        <v>-4.5999999999999996</v>
+      </c>
+      <c r="C40">
+        <v>-3</v>
+      </c>
+      <c r="D40">
+        <f t="shared" si="2"/>
+        <v>1.5999999999999996</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A41">
+        <v>3.1</v>
+      </c>
+      <c r="B41">
+        <v>-5.5</v>
+      </c>
+      <c r="C41">
+        <v>-4.2</v>
+      </c>
+      <c r="D41">
+        <f t="shared" si="2"/>
+        <v>1.2999999999999998</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A42">
+        <v>3.4</v>
+      </c>
+      <c r="B42">
+        <v>-4.6500000000000004</v>
+      </c>
+      <c r="C42">
+        <v>-3.2</v>
+      </c>
+      <c r="D42">
+        <f t="shared" si="2"/>
+        <v>1.4500000000000002</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A43">
+        <v>3.6</v>
+      </c>
+      <c r="B43">
+        <v>-5.3</v>
+      </c>
+      <c r="C43">
+        <v>-3.9</v>
+      </c>
+      <c r="D43">
         <f t="shared" si="2"/>
         <v>1.4</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A32">
-        <v>10.199999999999999</v>
-      </c>
-      <c r="B32">
-        <v>-4.9000000000000004</v>
-      </c>
-      <c r="C32">
-        <v>-4.1500000000000004</v>
-      </c>
-      <c r="D32">
-        <v>2.1</v>
-      </c>
-      <c r="E32">
-        <v>2.8</v>
-      </c>
-      <c r="F32">
-        <f t="shared" si="2"/>
-        <v>0.72499999999999987</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A33">
-        <v>11.2</v>
-      </c>
-      <c r="B33">
-        <v>8.25</v>
-      </c>
-      <c r="C33">
-        <v>8.9</v>
-      </c>
-      <c r="D33">
-        <v>2.1</v>
-      </c>
-      <c r="E33">
-        <v>2.6</v>
-      </c>
-      <c r="F33">
-        <f t="shared" si="2"/>
-        <v>0.57500000000000018</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A34">
-        <v>12.2</v>
-      </c>
-      <c r="B34">
-        <v>1.9</v>
-      </c>
-      <c r="C34">
-        <v>2.65</v>
-      </c>
-      <c r="D34">
-        <v>8.1999999999999993</v>
-      </c>
-      <c r="E34">
-        <v>8.9499999999999993</v>
-      </c>
-      <c r="F34">
-        <f t="shared" si="2"/>
-        <v>0.75000000000000022</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A35">
-        <v>2.2999999999999998</v>
-      </c>
-      <c r="F35">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A36">
-        <v>2.4</v>
-      </c>
-      <c r="F36">
-        <v>1.1000000000000001</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A37">
-        <v>2.6</v>
-      </c>
-      <c r="F37">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A38">
-        <v>2.8</v>
-      </c>
-      <c r="F38">
-        <v>1.3</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A39">
-        <v>2.9</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A40">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A41">
-        <v>3.1</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A42">
-        <v>3.4</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A43">
-        <v>3.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>